<commit_message>
EPC ortak adayları marka tercihleriyle; Huawei bölge yapısı ve garanti riski bölümü
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vs3tis47Aza7HeP1K6EeuU
</commit_message>
<xml_diff>
--- a/Maldivler_Potansiyel_Musteri_Listesi.xlsx
+++ b/Maldivler_Potansiyel_Musteri_Listesi.xlsx
@@ -264,14 +264,15 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Ortaklar" displayName="Ortaklar" ref="A1:E13" headerRowCount="1">
-  <autoFilter ref="A1:E13"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Ortaklar" displayName="Ortaklar" ref="A1:F14" headerRowCount="1">
+  <autoFilter ref="A1:F14"/>
+  <tableColumns count="6">
     <tableColumn id="1" name="Firma"/>
     <tableColumn id="2" name="Tür"/>
-    <tableColumn id="3" name="Neden uygun"/>
-    <tableColumn id="4" name="Web sitesi"/>
-    <tableColumn id="5" name="Not"/>
+    <tableColumn id="3" name="Bilinen marka tercihi (inverter/batarya)"/>
+    <tableColumn id="4" name="Karea / HYXI için değerlendirme"/>
+    <tableColumn id="5" name="Web sitesi"/>
+    <tableColumn id="6" name="Not"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -9270,14 +9271,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -9293,15 +9295,20 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Neden uygun</t>
+          <t>Bilinen marka tercihi (inverter/batarya)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>Karea / HYXI için değerlendirme</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
           <t>Web sitesi</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Not</t>
         </is>
@@ -9315,20 +9322,25 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>GES lideri / EPC</t>
+          <t>GES lideri / EPC (Avusturya, Malé'de yerleşik)</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>50+ resort müşterisi var; ESS ilavesi gereken GES'lerin çoğu onların. ESS tedarikçisi olarak yaklaşılabilir</t>
+          <t>Panel: kendi SolarSea sistemi. Batarya markası kamuya açık değil</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
+          <t>50+ resortta GES; Veligandu (1,7 MWh) ve RAH GILI (2,5 MWh) bataryalarını da kurdu. Batarya tedarikçisi olarak HYXI için en büyük potansiyel</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
           <t>swimsol.com</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Hem rakip hem müşteri olabilir</t>
         </is>
@@ -9337,268 +9349,318 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Ecogreen Maldives</t>
+          <t>Avi Technologies</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Yerel kurulumcu</t>
+          <t>Yerel EPC (2015)</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Tüm atollerde turnkey GES; yerel lisans ve saha ekibi</t>
+          <t>Kamuya açık marka bilgisi yok</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>ecogreenmaldives.com</t>
+          <t>GES + ESS + dizel entegrasyonu yapıyor (Haa Alif'te 14 adada 3,78 MWh ESS). 15+ MW kurulum. HYXI C&amp;I ESS için en uygun yerel ortak adayı</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Yerel ortak adayı</t>
+          <t>avitech.com.mv</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Yerel ortak – 1. öncelik</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Renewable Energy Maldives (REM)</t>
+          <t>Atoll Solar (Octopus Systems)</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Yerel kurulumcu</t>
+          <t>Yerel EPC, resort odaklı</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>2012'den beri yerel GES deneyimi</t>
+          <t>BYD ile çalışıyor</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Doğrulanmalı</t>
+          <t>Ana şirket Octopus Systems resortların sistem entegratörü, yani tüm resortlara zaten erişimi var. BYD'ye alternatif ikinci marka olarak HYXI sunulabilir</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Yerel ortak adayı</t>
+          <t>atollsolar.com</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Yerel ortak – 1. öncelik</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Avi Technologies</t>
+          <t>Ecogreen Maldives</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Kurulumcu</t>
+          <t>Yerel kurulumcu (2014)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Batarya entegrasyonu odaklı</t>
+          <t>Kamuya açık marka bilgisi yok</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Doğrulanmalı</t>
+          <t>Resort, misafirhane, konut ve tekne GES. Ağırlıklı olarak küçük/orta ölçek</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Ortak adayı</t>
+          <t>ecogreenmaldives.com</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Yerel ortak adayı</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Solar Atolls / Atoll Solar / AOI Utopia</t>
+          <t>Renewable Energy Maldives (REM)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Yerel kurulumcular</t>
+          <t>Yerel kurulumcu (2006)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ENF Solar dizininde Maldivler kurulumcuları</t>
+          <t>Sri Lanka kolu (REM Lanka) SolaX kullanıyor</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>enfsolar.com/directory/installer/Maldives</t>
+          <t>~25 ada ve resortlarla çalışmış eski oyuncu</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Ön eleme yapılmalı</t>
+          <t>LinkedIn: REM Solar</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Yerel ortak adayı</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Hayleys Fentons</t>
+          <t>SunCore Energy</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Bölgesel EPC (Sri Lanka)</t>
+          <t>Yerel GES firması</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Maldivler resort referansı (Sun Siyam) var; ürün tedarikçisi arıyor olabilir</t>
+          <t>Kamuya açık marka bilgisi yok</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>fentons.lk (doğrulanmalı)</t>
+          <t>16+ yıllık proje direktörü; kamu ve kurumsal projeler</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Ortak veya rakip</t>
+          <t>suncore.mv</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Yerel ortak adayı</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Canopy Power</t>
+          <t>Hayleys Fentons / Hayleys Solar</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Mikro şebeke EPC (Singapur)</t>
+          <t>Bölgesel EPC (Sri Lanka, 500+ MW)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Resort mikro şebeke uzmanı; Huawei ile çalışıyor</t>
+          <t>HUAWEI kullanıyor (inverter tedarikçileri arasında; Hayleys Electronics Huawei ile ortak forum yaptı); BYD batarya ortağı</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>canopypower.com</t>
+          <t>Sun Siyam projesinin yüklenicisi. Huawei kanalında oldukları için HYXI'ye geçmeleri zor; Huawei tarafında ise bölgesel rakip/kanal</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Huawei kanalı ile çakışma kontrol edilmeli</t>
+          <t>hayleysfentons.com</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Huawei kullanıcısı</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Resort jeneratör bakım/servis firmaları</t>
+          <t>Canopy Power</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>O&amp;M</t>
+          <t>Mikro şebeke EPC (Singapur)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Her resortun enerji santraline zaten erişimleri var; hibrit kontrol entegrasyonu için kritik</t>
+          <t>HUAWEI ESS (Soneva Secret 3 MWh)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Saha ziyaretinde tespit edilecek</t>
+          <t>Huawei kanalında</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Cummins, MTU, Caterpillar yerel bayileri</t>
+          <t>canopypower.com</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Huawei kullanıcısı</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>SunCore Energy</t>
+          <t>Solmacher Solar Energy</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Yerel GES firması (Maldivler)</t>
+          <t>EPC</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Maldivli GES şirketi; 16+ yıllık proje yöneticisi var</t>
+          <t>HUAWEI (Royal Rosewood 40 MWh ESS + inverter, Ağu. 2026)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>suncore.mv</t>
+          <t>Huawei'nin Maldivler'deki en büyük projesi bu firmada</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Yerel ortak adayı</t>
+          <t>Doğrulanmalı</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Huawei kullanıcısı</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Atoll Solar</t>
+          <t>SINOSOAR</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Yerel GES / yüzer GES</t>
+          <t>Çin EPC – kamu hibrit projeleri</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Hotelier Maldives GM Forum 2026'da Ocean Sun ile lagün yüzer GES sunumu yaptı – resort yöneticilerine erişimi var</t>
+          <t>Kendi PCS/EMS'i; Sungrow ile bağlantılı</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Doğrulanmalı</t>
+          <t>134 adada kamu mikro şebeke projesi (ADB/ASSURE 40 MWh dahil). Kamu ihaleleri tarafında güçlü rakip</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Yerel ortak adayı</t>
+          <t>sinosoarhybrid.com</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Rakip (kamu)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>DEIF</t>
+          <t>Resort jeneratör bakım/servis firmaları</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Hibrit kontrol sistemi (Danimarka)</t>
+          <t>O&amp;M</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Maldivler'de bir lüks resortta dizel+GES+batarya hibrit kontrolünü yaptı; ESS entegrasyonunda teknik ortak</t>
+          <t>Cummins, MTU, Caterpillar yerel bayileri</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>deif.com</t>
+          <t>Her resortun enerji santraline zaten erişimleri var; hibrit kontrol entegrasyonu için kritik</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Saha ziyaretinde tespit edilecek</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Teknik ortak</t>
         </is>
@@ -9607,25 +9669,62 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>DEIF</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Hibrit kontrol sistemi (Danimarka)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Maldivler'de bir lüks resortta dizel+GES+batarya kontrolünü yaptı; ESS entegrasyonunda teknik ortak</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>deif.com</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Teknik ortak</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
           <t>Elemental Water Makers</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Güneş enerjili su arıtma</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Resortlarda tuzdan arındırma en büyük elektrik yüklerinden biri</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>elementalwatermakers.com</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Tamamlayıcı ortak</t>
         </is>

</xml_diff>

<commit_message>
Mail takibi: 2. tur (grup merkezleri ve büyük resortlar) işlendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vs3tis47Aza7HeP1K6EeuU
</commit_message>
<xml_diff>
--- a/Maldivler_Potansiyel_Musteri_Listesi.xlsx
+++ b/Maldivler_Potansiyel_Musteri_Listesi.xlsx
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1362,36 +1362,506 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Villa Hotels &amp; Resorts (Villa Group)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – grup merkezi</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>sales@villaresorts.com</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – battery storage for Villa Park's existing solar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Crown &amp; Champa Resorts</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – grup merkezi</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>info@crownandchamparesorts.com</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for your next resorts after Veligandu</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Atmosphere Core</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – grup merkezi</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>info@atmospherecore.com</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Technical Services – battery storage for your resorts and Amaraa Faru</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Sun Siyam Resorts</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – grup merkezi</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>sales@sunsiyam.com</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – next phase of your 2030 renewable target</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Adaaran / Aitken Spence (Malé ofisi)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – grup merkezi</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>inquiries.mv@adaaran.com.mv</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – reducing diesel costs at your Maldives resorts</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Cinnamon Hotels – John Keells Maldivian Resorts</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – grup merkezi</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>sales.mv@cinnamonhotels.com</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for your Maldives resorts</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>CROSSROADS Maldives (Singha Estate)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – grup merkezi</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>sales@crossroadsmaldives.com</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for the CROSSROADS islands</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Kandima / Pulse Hotels &amp; Resorts</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – grup merkezi</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>KeepinTouch@pulseresorts.com</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Kandima Maldives</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Meeru Maldives Resort Island</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>reservations@meeru.com</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Chief Engineer – solar and storage for Meeru</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2. tur</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Canareef Resort Maldives</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>info@canareef.com</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – battery storage for your rooftop solar</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Renkler:</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>Mail gönderildi</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Yanıt geldi</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>Görüşme planlandı</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>İlgilenmiyor</t>
         </is>
@@ -1903,68 +2373,68 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Canareef Resort Maldives</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Addu</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Bağımsız</t>
         </is>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="5" t="n">
         <v>280</v>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Kısmi GES, ESS yok/bilinmiyor</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Büyük çatı GES kurulumu duyuruldu</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>canareef.com</t>
         </is>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>info@canareef.com</t>
         </is>
       </c>
-      <c r="J7" s="11" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>+960 689 6677</t>
         </is>
       </c>
-      <c r="K7" s="11" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L7" s="11" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
         <is>
           <t>https://canareef.com/contact-us/</t>
         </is>
       </c>
-      <c r="M7" s="11" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N7" s="11" t="n">
+      <c r="N7" s="5" t="n">
         <v>6</v>
       </c>
       <c r="O7" s="12" t="inlineStr">
@@ -1972,9 +2442,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="P7" s="11" t="inlineStr">
+      <c r="P7" s="5" t="inlineStr">
         <is>
           <t>büyük resort (yüksek dizel tüketimi); GES var ama ESS yok -&gt; en uygun ESS ilavesi hedefi</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -2131,68 +2606,68 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Kandima Maldives</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Dhaalu</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Pulse Hotels &amp; Resorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="5" t="n">
         <v>266</v>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>kandima.com</t>
         </is>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>mykindofplace@kandima.com; reservations@kandima.com</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>+960 676 0077</t>
         </is>
       </c>
-      <c r="K10" s="11" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Otel rehberi / arama sonucu</t>
         </is>
       </c>
-      <c r="L10" s="11" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>https://www.maldivesyp.com/company/638/Kandima_Maldives</t>
         </is>
       </c>
-      <c r="M10" s="11" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N10" s="11" t="n">
+      <c r="N10" s="5" t="n">
         <v>6</v>
       </c>
       <c r="O10" s="12" t="inlineStr">
@@ -2200,9 +2675,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="P10" s="11" t="inlineStr">
+      <c r="P10" s="5" t="inlineStr">
         <is>
           <t>büyük resort (yüksek dizel tüketimi); bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -4113,68 +4593,68 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="n">
+      <c r="A36" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Meeru Maldives Resort Island</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Bağımsız (Maldivli)</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
+      <c r="E36" s="5" t="n">
         <v>286</v>
       </c>
-      <c r="F36" s="11" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G36" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="11" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>meeru.com</t>
         </is>
       </c>
-      <c r="I36" s="11" t="inlineStr">
+      <c r="I36" s="5" t="inlineStr">
         <is>
           <t>reservations@meeru.com</t>
         </is>
       </c>
-      <c r="J36" s="11" t="inlineStr">
+      <c r="J36" s="5" t="inlineStr">
         <is>
           <t>+960 664 3157</t>
         </is>
       </c>
-      <c r="K36" s="11" t="inlineStr">
+      <c r="K36" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L36" s="11" t="inlineStr">
+      <c r="L36" s="5" t="inlineStr">
         <is>
           <t>https://www.meeru.com/one-island-one-resort-contact-us/</t>
         </is>
       </c>
-      <c r="M36" s="11" t="inlineStr">
+      <c r="M36" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N36" s="11" t="n">
+      <c r="N36" s="5" t="n">
         <v>5</v>
       </c>
       <c r="O36" s="13" t="inlineStr">
@@ -4182,9 +4662,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P36" s="11" t="inlineStr">
+      <c r="P36" s="5" t="inlineStr">
         <is>
           <t>büyük resort (yüksek dizel tüketimi); bilinen GES yok -&gt; GES+ESS paketi</t>
+        </is>
+      </c>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -8531,32 +9016,32 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Villa Hotels &amp; Resorts (Villa Group)</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Malé (Maldivli)</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>5+</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Villa Park (eski Sun Island), Villa Nautica (eski Paradise Island), Royal Island</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Büyük, orta segment; Villa Park'ta 2.400+ panel var, batarya bilgisi yok</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>villaresorts.com</t>
         </is>
@@ -8566,54 +9051,59 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>hello@villaresorts.com; sales@villaresorts.com</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>+960 334 4777</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Villa House, Kandi Dhonmanik Goalhi, Malé 20181</t>
         </is>
       </c>
-      <c r="K3" s="11" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>https://villaresorts.com/contact/</t>
         </is>
       </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Sun Siyam Resorts</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Malé (Maldivli)</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Siyam World, Olhuveli, Iru Fushi, Iru Veli, Vilu Reef</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>2 resortta GES+ESS (Hayleys Fentons); %50 yenilenebilir @2030 hedefi -&gt; kalan 3 resort için 2. faz</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>sunsiyam.com</t>
         </is>
@@ -8623,54 +9113,59 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>sales@sunsiyam.com; book@sunsiyam.com</t>
         </is>
       </c>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>+960 332 5977</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Sun Siyam Building, Boduthakurufaanu Magu, Malé 20066</t>
         </is>
       </c>
-      <c r="K4" s="11" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>https://prelive.sunsiyam.com/contact/</t>
         </is>
       </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Crown &amp; Champa Resorts</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Malé (Maldivli)</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Kuredu, Komandoo, Veligandu, Hurawalhi, Kudadoo, Vilamendhoo, Meeru (doğrulanmalı)</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Veligandu tamamlandı; Kuredu (380 oda) en büyük fırsat</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>crownandchamparesorts.com</t>
         </is>
@@ -8680,24 +9175,29 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>info@crownandchamparesorts.com</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>+960 664 0219</t>
         </is>
       </c>
-      <c r="J5" s="11" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Champa Building 3. kat, Kandi Dhon Manik Goalhi, Malé 20187</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>https://www.crownandchamparesorts.com/inquire-now.html</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -8759,32 +9259,32 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Atmosphere Core</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Malé / Hindistan</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>9-10</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Kanifushi, OZEN Reserve, OZEN LIFE, VARU, Amaraa Faru (2027)</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Çatı GES yaygın; ESS ilavesi ve yeni açılışlar fırsat</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>atmospherecore.com</t>
         </is>
@@ -8794,24 +9294,29 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>info@atmospherecore.com</t>
         </is>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>+960 330 0668</t>
         </is>
       </c>
-      <c r="J7" s="11" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Boduthakurufaanu Magu, Malé 20094</t>
         </is>
       </c>
-      <c r="K7" s="11" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>https://www.atmospherecore.com/contact-us</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -8878,32 +9383,32 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Aitken Spence (Adaaran / Heritance)</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Colombo, Sri Lanka</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Adaaran Hudhuranfushi, Rannalhi, Vadoo, Heritance Aarah</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Kamuya açık GES bilgisi sınırlı</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>aitkenspencehotels.com</t>
         </is>
@@ -8913,54 +9418,59 @@
           <t>B</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>inquiries.mv@adaaran.com.mv</t>
         </is>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>+960 664 0375</t>
         </is>
       </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>H. Thuniya 6. kat, Boduthakurufaanu Magu, Malé 20026</t>
         </is>
       </c>
-      <c r="K9" s="11" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>https://www.aitkenspencehotels.com/contact-us.html</t>
         </is>
       </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Cinnamon Hotels (John Keells)</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Colombo, Sri Lanka</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Dhonveli, Velifushi, Ellaidhoo, Hakuraa</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Kamuya açık GES bilgisi sınırlı</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>cinnamonhotels.com</t>
         </is>
@@ -8970,24 +9480,29 @@
           <t>B</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>sales.mv@cinnamonhotels.com</t>
         </is>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>+960 333 6000</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>H. Maizan Building 2. kat, Sosun Magu, Malé 20252</t>
         </is>
       </c>
-      <c r="K10" s="11" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>https://www.maldivesyp.com/company/547/Cinnamon_Dhonveli_Maldives</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -9049,32 +9564,32 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Pulse Hotels &amp; Resorts (Kandima)</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Malé / Singapur</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>1-2</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Kandima</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Kamuya açık GES bilgisi yok. Mayıs 2026'da Director of Engineering ilanı açtı (yeni kişi göreve başlamış olabilir)</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>kandima.com</t>
         </is>
@@ -9084,54 +9599,59 @@
           <t>B</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>KeepinTouch@pulseresorts.com</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>+65 6838 9123 (Singapur)</t>
         </is>
       </c>
-      <c r="J12" s="11" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Kaneeru Villa 4. kat, Orchid Magu, Malé 20212</t>
         </is>
       </c>
-      <c r="K12" s="11" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>https://kandima.com/en/explore/contact</t>
         </is>
       </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>CROSSROADS / Singha Estate</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Bangkok, Tayland</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>2 + marina</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Hard Rock, SAii Lagoon</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Entegre ada kompleksi, tek enerji santrali</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>crossroadsmaldives.com</t>
         </is>
@@ -9141,24 +9661,29 @@
           <t>B</t>
         </is>
       </c>
-      <c r="H13" s="11" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>sales@crossroadsmaldives.com</t>
         </is>
       </c>
-      <c r="I13" s="11" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>+960 665 1200</t>
         </is>
       </c>
-      <c r="J13" s="11" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>South Malé Atoll, P.O. Box 2097</t>
         </is>
       </c>
-      <c r="K13" s="11" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>https://crossroadsmaldives.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mail takibi: 4. tur (31-59) işlendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vs3tis47Aza7HeP1K6EeuU
</commit_message>
<xml_diff>
--- a/Maldivler_Potansiyel_Musteri_Listesi.xlsx
+++ b/Maldivler_Potansiyel_Musteri_Listesi.xlsx
@@ -831,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2302,36 +2302,1399 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Anantara Kihavah Maldives Villas</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>kihavahmaldives@anantara.com</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Anantara Kihavah</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Sheraton Maldives Full Moon</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>sheraton.maldives@sheraton.com</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Sheraton Maldives Full Moon</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Six Senses Laamu</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>reservations-laamu@sixsenses.com</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Six Senses Laamu</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Six Senses Kanuhura</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>reservations-maldives@sixsenses.com</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Six Senses Kanuhura</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Dusit Thani Maldives</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>resmaldives@dusit.com</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Dusit Thani Maldives</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Grand Park Kodhipparu</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>info@grandparkkodhipparu.com</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Grand Park Kodhipparu</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>InterContinental Maldives Maamunagau</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Intercontinental.Maldives@ihg.com</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for InterContinental Maldives Maamunagau</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Summer Island Maldives</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>reservations@summerislandmaldives.com</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Summer Island Maldives</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Embudu Village</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>sales@embuduvillage.com</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Embudu Village</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Biyadhoo Island Resort</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>biyadhoo@sunland.com.mv</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Biyadhoo Island Resort</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Malahini Kuda Bandos</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>reservations@malahini.mv</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Malahini Kuda Bandos</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>NH Collection Maldives Reethi</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>reethi@nhcollection.com</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for NH Collection Maldives Reethi</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Gili Lankanfushi</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>mr.friday@gili-lankanfushi.com</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Gili Lankanfushi</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Baros Maldives (VERSA)</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>reservations@baros.com</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Baros Maldives</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Milaidhoo Maldives (VERSA)</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>welcome@milaidhoo.com</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Milaidhoo Maldives</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Kandolhu Maldives (VERSA)</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>info@kandolhu.com</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Kandolhu Maldives</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Angsana Velavaru</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>reservations-velavaru@angsana.com</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Angsana Velavaru</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Club Med Kani &amp; Finolhu Villas</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>contactus.asia@clubmed.com</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Club Med Kani and Finolhu Villas</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Centara Maldives (Ras Fushi, Machchafushi, Mirage Lagoon)</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>crf@chr.co.th</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Centara Maldives</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Fairmont Maldives Sirru Fen Fushi</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>reservations@sirrufenfushi.com</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Sirru Fen Fushi</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Lily Beach Resort &amp; Spa</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>reservations@lilybeachmaldives.com</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Lily Beach Resort</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Radisson Blu Resort Maldives</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>info.maldives@radisson.com</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Radisson Blu Resort Maldives</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Pullman Maldives Maamutaa</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>H9924-re@accor.com</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Pullman Maldives Maamutaa</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Mercure Maldives Kooddoo</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>H9923@accor.com</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Mercure Maldives Kooddoo</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>OUTRIGGER Maldives Maafushivaru</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>maldives.maafushivaru@outrigger.com</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for OUTRIGGER Maldives Maafushivaru</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Hideaway Beach Resort &amp; Spa</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>reservations@hideawaybeachmaldives.com</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Hideaway Beach Resort</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>The Westin Maldives Miriandhoo</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>mlewi.reservation@westinhotels.com</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for The Westin Maldives Miriandhoo</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>JW Marriott Maldives Resort &amp; Spa</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>jwmaldivesreservations@marriott.com</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for JW Marriott Maldives</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>4. tur</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Jumeirah Maldives Olhahali Island</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Son kullanıcı – resort</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>reservations@jumeirah.com</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Attn: Engineering – solar and storage for Jumeirah Maldives Olhahali Island</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>Yanıt yoksa nazik hatırlatma maili</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>Renkler:</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
         <is>
           <t>Mail gönderildi</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
         <is>
           <t>Yanıt geldi</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="9" t="inlineStr">
         <is>
           <t>Görüşme planlandı</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>İlgilenmiyor</t>
         </is>
@@ -2934,68 +4297,68 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Club Med Kani</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Club Med</t>
         </is>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="5" t="n">
         <v>250</v>
       </c>
-      <c r="F8" s="12" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>clubmed.com</t>
         </is>
       </c>
-      <c r="I8" s="12" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J8" s="12" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>+960 664 3152</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>E-posta sayfada gizlenmiş; Club Med merkezi üzerinden</t>
         </is>
       </c>
-      <c r="L8" s="12" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>https://www.hotelcontact.net/club-med-kani-maldives-north-male-en.html</t>
         </is>
       </c>
-      <c r="M8" s="12" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N8" s="12" t="n">
+      <c r="N8" s="5" t="n">
         <v>6</v>
       </c>
       <c r="O8" s="11" t="inlineStr">
@@ -3003,9 +4366,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="P8" s="12" t="inlineStr">
+      <c r="P8" s="5" t="inlineStr">
         <is>
           <t>büyük resort (yüksek dizel tüketimi); bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -4176,68 +5544,68 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Centara Grand Island Resort</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Alif Dhaal (Güney Ari)</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Centara Hotels</t>
         </is>
       </c>
-      <c r="E24" s="12" t="n">
+      <c r="E24" s="5" t="n">
         <v>112</v>
       </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>Kısmi GES, ESS yok/bilinmiyor</t>
         </is>
       </c>
-      <c r="G24" s="12" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Yeni adı Machchafushi Island Resort (Centara Collection); tüm çatılarda GES</t>
         </is>
       </c>
-      <c r="H24" s="12" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>centarahotelsresorts.com</t>
         </is>
       </c>
-      <c r="I24" s="12" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J24" s="12" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>+960 668 8000</t>
         </is>
       </c>
-      <c r="K24" s="12" t="inlineStr">
+      <c r="K24" s="5" t="inlineStr">
         <is>
           <t>NOT: Yeni adı 'Machchafushi Island Resort &amp; Spa, The Centara Collection'; e-posta sayfada gizlenmiş</t>
         </is>
       </c>
-      <c r="L24" s="12" t="inlineStr">
+      <c r="L24" s="5" t="inlineStr">
         <is>
           <t>https://www.centarahotelsresorts.com/centaragrand/cirm/contact/</t>
         </is>
       </c>
-      <c r="M24" s="12" t="inlineStr">
+      <c r="M24" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N24" s="12" t="n">
+      <c r="N24" s="5" t="n">
         <v>5</v>
       </c>
       <c r="O24" s="13" t="inlineStr">
@@ -4245,75 +5613,80 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P24" s="12" t="inlineStr">
+      <c r="P24" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; GES var ama ESS yok -&gt; en uygun ESS ilavesi hedefi; çok-resortlu grup (tek kararla birden fazla ada)</t>
         </is>
       </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n">
+      <c r="A25" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Centara Ras Fushi</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Centara Hotels</t>
         </is>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E25" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G25" s="12" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H25" s="12" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>centarahotelsresorts.com</t>
         </is>
       </c>
-      <c r="I25" s="12" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>crf@chr.co.th</t>
         </is>
       </c>
-      <c r="J25" s="12" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>+960 664 3880</t>
         </is>
       </c>
-      <c r="K25" s="12" t="inlineStr">
+      <c r="K25" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L25" s="12" t="inlineStr">
+      <c r="L25" s="5" t="inlineStr">
         <is>
           <t>https://www.centarahotelsresorts.com/centara/CRF/contact</t>
         </is>
       </c>
-      <c r="M25" s="12" t="inlineStr">
+      <c r="M25" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N25" s="12" t="n">
+      <c r="N25" s="5" t="n">
         <v>5</v>
       </c>
       <c r="O25" s="13" t="inlineStr">
@@ -4321,9 +5694,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P25" s="12" t="inlineStr">
+      <c r="P25" s="5" t="inlineStr">
         <is>
           <t>orta-büyük resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -5723,68 +7101,68 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="n">
+      <c r="A44" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>Sheraton Maldives Full Moon</t>
         </is>
       </c>
-      <c r="C44" s="12" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D44" s="12" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Marriott markası</t>
         </is>
       </c>
-      <c r="E44" s="12" t="n">
+      <c r="E44" s="5" t="n">
         <v>176</v>
       </c>
-      <c r="F44" s="12" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G44" s="12" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H44" s="12" t="inlineStr">
+      <c r="H44" s="5" t="inlineStr">
         <is>
           <t>marriott.com</t>
         </is>
       </c>
-      <c r="I44" s="12" t="inlineStr">
+      <c r="I44" s="5" t="inlineStr">
         <is>
           <t>sheraton.maldives@sheraton.com</t>
         </is>
       </c>
-      <c r="J44" s="12" t="inlineStr">
+      <c r="J44" s="5" t="inlineStr">
         <is>
           <t>+960 664 2010</t>
         </is>
       </c>
-      <c r="K44" s="12" t="inlineStr">
+      <c r="K44" s="5" t="inlineStr">
         <is>
           <t>Otel rehberi / arama sonucu</t>
         </is>
       </c>
-      <c r="L44" s="12" t="inlineStr">
+      <c r="L44" s="5" t="inlineStr">
         <is>
           <t>https://www.hotelcontact.net/sheraton-maldives-full-moon-resort-spa-vihamanaafushi-en.html</t>
         </is>
       </c>
-      <c r="M44" s="12" t="inlineStr">
+      <c r="M44" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N44" s="12" t="n">
+      <c r="N44" s="5" t="n">
         <v>5</v>
       </c>
       <c r="O44" s="13" t="inlineStr">
@@ -5792,75 +7170,80 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P44" s="12" t="inlineStr">
+      <c r="P44" s="5" t="inlineStr">
         <is>
           <t>orta-büyük resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
         </is>
       </c>
+      <c r="Q44" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="12" t="n">
+      <c r="A45" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Six Senses Laamu</t>
         </is>
       </c>
-      <c r="C45" s="12" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>Laamu</t>
         </is>
       </c>
-      <c r="D45" s="12" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>Six Senses (IHG)</t>
         </is>
       </c>
-      <c r="E45" s="12" t="n">
+      <c r="E45" s="5" t="n">
         <v>97</v>
       </c>
-      <c r="F45" s="12" t="inlineStr">
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t>Kısmi GES, ESS yok/bilinmiyor</t>
         </is>
       </c>
-      <c r="G45" s="12" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>Sürdürülebilirlik odaklı; GES bilgisi var, kapsamı doğrulanmalı</t>
         </is>
       </c>
-      <c r="H45" s="12" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>sixsenses.com</t>
         </is>
       </c>
-      <c r="I45" s="12" t="inlineStr">
+      <c r="I45" s="5" t="inlineStr">
         <is>
           <t>reservations-laamu@sixsenses.com</t>
         </is>
       </c>
-      <c r="J45" s="12" t="inlineStr">
+      <c r="J45" s="5" t="inlineStr">
         <is>
           <t>+960 680 0800</t>
         </is>
       </c>
-      <c r="K45" s="12" t="inlineStr">
+      <c r="K45" s="5" t="inlineStr">
         <is>
           <t>Arama sonucu</t>
         </is>
       </c>
-      <c r="L45" s="12" t="inlineStr">
+      <c r="L45" s="5" t="inlineStr">
         <is>
           <t>https://wetu.com/iBrochure/en/Information/63679/six_senses_laamu/Contact</t>
         </is>
       </c>
-      <c r="M45" s="12" t="inlineStr">
+      <c r="M45" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N45" s="12" t="n">
+      <c r="N45" s="5" t="n">
         <v>5</v>
       </c>
       <c r="O45" s="13" t="inlineStr">
@@ -5868,9 +7251,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P45" s="12" t="inlineStr">
+      <c r="P45" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; GES var ama ESS yok -&gt; en uygun ESS ilavesi hedefi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -6495,68 +7883,68 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="n">
+      <c r="A54" s="5" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="12" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Anantara Kihavah</t>
         </is>
       </c>
-      <c r="C54" s="12" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Baa</t>
         </is>
       </c>
-      <c r="D54" s="12" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Minor Hotels</t>
         </is>
       </c>
-      <c r="E54" s="12" t="n">
+      <c r="E54" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="F54" s="12" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G54" s="12" t="inlineStr">
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H54" s="12" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>anantara.com</t>
         </is>
       </c>
-      <c r="I54" s="12" t="inlineStr">
+      <c r="I54" s="5" t="inlineStr">
         <is>
           <t>kihavahmaldives@anantara.com</t>
         </is>
       </c>
-      <c r="J54" s="12" t="inlineStr">
+      <c r="J54" s="5" t="inlineStr">
         <is>
           <t>+960 660 1020</t>
         </is>
       </c>
-      <c r="K54" s="12" t="inlineStr">
+      <c r="K54" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L54" s="12" t="inlineStr">
+      <c r="L54" s="5" t="inlineStr">
         <is>
           <t>https://www.anantara.com/en/kihavah-maldives/contact</t>
         </is>
       </c>
-      <c r="M54" s="12" t="inlineStr">
+      <c r="M54" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N54" s="12" t="n">
+      <c r="N54" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O54" s="13" t="inlineStr">
@@ -6564,75 +7952,80 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P54" s="12" t="inlineStr">
+      <c r="P54" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
         </is>
       </c>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="12" t="n">
+      <c r="A55" s="5" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Angsana Velavaru</t>
         </is>
       </c>
-      <c r="C55" s="12" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Dhaalu</t>
         </is>
       </c>
-      <c r="D55" s="12" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>Banyan Group</t>
         </is>
       </c>
-      <c r="E55" s="12" t="n">
+      <c r="E55" s="5" t="n">
         <v>113</v>
       </c>
-      <c r="F55" s="12" t="inlineStr">
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G55" s="12" t="inlineStr">
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H55" s="12" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>angsana.com</t>
         </is>
       </c>
-      <c r="I55" s="12" t="inlineStr">
+      <c r="I55" s="5" t="inlineStr">
         <is>
           <t>reservations-velavaru@angsana.com</t>
         </is>
       </c>
-      <c r="J55" s="12" t="inlineStr">
+      <c r="J55" s="5" t="inlineStr">
         <is>
           <t>+960 676 0028</t>
         </is>
       </c>
-      <c r="K55" s="12" t="inlineStr">
+      <c r="K55" s="5" t="inlineStr">
         <is>
           <t>Arama sonucu</t>
         </is>
       </c>
-      <c r="L55" s="12" t="inlineStr">
+      <c r="L55" s="5" t="inlineStr">
         <is>
           <t>https://www.angsana.com/maldives/velavaru/travel-information</t>
         </is>
       </c>
-      <c r="M55" s="12" t="inlineStr">
+      <c r="M55" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N55" s="12" t="n">
+      <c r="N55" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O55" s="13" t="inlineStr">
@@ -6640,9 +8033,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P55" s="12" t="inlineStr">
+      <c r="P55" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q55" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -6725,68 +8123,68 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="n">
+      <c r="A57" s="5" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>Baros Maldives</t>
         </is>
       </c>
-      <c r="C57" s="12" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D57" s="12" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>VERSA Hospitality</t>
         </is>
       </c>
-      <c r="E57" s="12" t="n">
+      <c r="E57" s="5" t="n">
         <v>75</v>
       </c>
-      <c r="F57" s="12" t="inlineStr">
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G57" s="12" t="inlineStr">
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H57" s="12" t="inlineStr">
+      <c r="H57" s="5" t="inlineStr">
         <is>
           <t>baros.com</t>
         </is>
       </c>
-      <c r="I57" s="12" t="inlineStr">
+      <c r="I57" s="5" t="inlineStr">
         <is>
           <t>reservations@baros.com</t>
         </is>
       </c>
-      <c r="J57" s="12" t="inlineStr">
+      <c r="J57" s="5" t="inlineStr">
         <is>
           <t>+960 664 2672</t>
         </is>
       </c>
-      <c r="K57" s="12" t="inlineStr">
+      <c r="K57" s="5" t="inlineStr">
         <is>
           <t>Arama sonucu (otel sitesi)</t>
         </is>
       </c>
-      <c r="L57" s="12" t="inlineStr">
+      <c r="L57" s="5" t="inlineStr">
         <is>
           <t>https://barosthn.emarketingeye.net/contact-us</t>
         </is>
       </c>
-      <c r="M57" s="12" t="inlineStr">
+      <c r="M57" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N57" s="12" t="n">
+      <c r="N57" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O57" s="13" t="inlineStr">
@@ -6794,9 +8192,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P57" s="12" t="inlineStr">
+      <c r="P57" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q57" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -6953,68 +8356,68 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="n">
+      <c r="A60" s="5" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="12" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>Club Med Finolhu Villas</t>
         </is>
       </c>
-      <c r="C60" s="12" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D60" s="12" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>Club Med</t>
         </is>
       </c>
-      <c r="E60" s="12" t="n">
+      <c r="E60" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="F60" s="12" t="inlineStr">
+      <c r="F60" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G60" s="12" t="inlineStr">
+      <c r="G60" s="5" t="inlineStr">
         <is>
           <t>Kani ile aynı lagün</t>
         </is>
       </c>
-      <c r="H60" s="12" t="inlineStr">
+      <c r="H60" s="5" t="inlineStr">
         <is>
           <t>clubmed.com</t>
         </is>
       </c>
-      <c r="I60" s="12" t="inlineStr">
+      <c r="I60" s="5" t="inlineStr">
         <is>
           <t>contactus.asia@clubmed.com (bölge merkezi)</t>
         </is>
       </c>
-      <c r="J60" s="12" t="inlineStr">
+      <c r="J60" s="5" t="inlineStr">
         <is>
           <t>+960 664 4040</t>
         </is>
       </c>
-      <c r="K60" s="12" t="inlineStr">
+      <c r="K60" s="5" t="inlineStr">
         <is>
           <t>Club Med sitesi</t>
         </is>
       </c>
-      <c r="L60" s="12" t="inlineStr">
+      <c r="L60" s="5" t="inlineStr">
         <is>
           <t>https://www.clubmed.us/r/the-finolhu-villas/y</t>
         </is>
       </c>
-      <c r="M60" s="12" t="inlineStr">
+      <c r="M60" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N60" s="12" t="n">
+      <c r="N60" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O60" s="13" t="inlineStr">
@@ -7022,9 +8425,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P60" s="12" t="inlineStr">
+      <c r="P60" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q60" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -7107,68 +8515,68 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="n">
+      <c r="A62" s="5" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="12" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>Dusit Thani Maldives</t>
         </is>
       </c>
-      <c r="C62" s="12" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>Baa</t>
         </is>
       </c>
-      <c r="D62" s="12" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>Dusit</t>
         </is>
       </c>
-      <c r="E62" s="12" t="n">
+      <c r="E62" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="F62" s="12" t="inlineStr">
+      <c r="F62" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G62" s="12" t="inlineStr">
+      <c r="G62" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H62" s="12" t="inlineStr">
+      <c r="H62" s="5" t="inlineStr">
         <is>
           <t>dusit.com</t>
         </is>
       </c>
-      <c r="I62" s="12" t="inlineStr">
+      <c r="I62" s="5" t="inlineStr">
         <is>
           <t>resmaldives@dusit.com</t>
         </is>
       </c>
-      <c r="J62" s="12" t="inlineStr">
+      <c r="J62" s="5" t="inlineStr">
         <is>
           <t>+960 660 8888</t>
         </is>
       </c>
-      <c r="K62" s="12" t="inlineStr">
+      <c r="K62" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L62" s="12" t="inlineStr">
+      <c r="L62" s="5" t="inlineStr">
         <is>
           <t>https://www.dusit.com/dusitthani-maldives/contact-us/</t>
         </is>
       </c>
-      <c r="M62" s="12" t="inlineStr">
+      <c r="M62" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N62" s="12" t="n">
+      <c r="N62" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O62" s="13" t="inlineStr">
@@ -7176,9 +8584,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P62" s="12" t="inlineStr">
+      <c r="P62" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q62" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -7259,68 +8672,68 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="12" t="n">
+      <c r="A64" s="5" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="12" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>Embudu Village</t>
         </is>
       </c>
-      <c r="C64" s="12" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Güney Malé)</t>
         </is>
       </c>
-      <c r="D64" s="12" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>Bağımsız</t>
         </is>
       </c>
-      <c r="E64" s="12" t="n">
+      <c r="E64" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="F64" s="12" t="inlineStr">
+      <c r="F64" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G64" s="12" t="inlineStr">
+      <c r="G64" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H64" s="12" t="inlineStr">
+      <c r="H64" s="5" t="inlineStr">
         <is>
           <t>embudu.com</t>
         </is>
       </c>
-      <c r="I64" s="12" t="inlineStr">
+      <c r="I64" s="5" t="inlineStr">
         <is>
           <t>sales@embuduvillage.com</t>
         </is>
       </c>
-      <c r="J64" s="12" t="inlineStr">
+      <c r="J64" s="5" t="inlineStr">
         <is>
           <t>+960 664 4776</t>
         </is>
       </c>
-      <c r="K64" s="12" t="inlineStr">
+      <c r="K64" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L64" s="12" t="inlineStr">
+      <c r="L64" s="5" t="inlineStr">
         <is>
           <t>https://www.embuduvillage.com/contact-us</t>
         </is>
       </c>
-      <c r="M64" s="12" t="inlineStr">
+      <c r="M64" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N64" s="12" t="n">
+      <c r="N64" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O64" s="13" t="inlineStr">
@@ -7328,9 +8741,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P64" s="12" t="inlineStr">
+      <c r="P64" s="5" t="inlineStr">
         <is>
           <t>orta-büyük resort; bilinen GES yok -&gt; GES+ESS paketi</t>
+        </is>
+      </c>
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -7573,68 +8991,68 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="12" t="n">
+      <c r="A68" s="5" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="12" t="inlineStr">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>Gili Lankanfushi</t>
         </is>
       </c>
-      <c r="C68" s="12" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D68" s="12" t="inlineStr">
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>Bağımsız</t>
         </is>
       </c>
-      <c r="E68" s="12" t="n">
+      <c r="E68" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="F68" s="12" t="inlineStr">
+      <c r="F68" s="5" t="inlineStr">
         <is>
           <t>Kısmi GES, ESS yok/bilinmiyor</t>
         </is>
       </c>
-      <c r="G68" s="12" t="inlineStr">
+      <c r="G68" s="5" t="inlineStr">
         <is>
           <t>GES bilgisi var, kapsamı doğrulanmalı</t>
         </is>
       </c>
-      <c r="H68" s="12" t="inlineStr">
+      <c r="H68" s="5" t="inlineStr">
         <is>
           <t>gili-lankanfushi.com</t>
         </is>
       </c>
-      <c r="I68" s="12" t="inlineStr">
+      <c r="I68" s="5" t="inlineStr">
         <is>
           <t>mr.friday@gili-lankanfushi.com</t>
         </is>
       </c>
-      <c r="J68" s="12" t="inlineStr">
+      <c r="J68" s="5" t="inlineStr">
         <is>
           <t>+960 664 0304</t>
         </is>
       </c>
-      <c r="K68" s="12" t="inlineStr">
+      <c r="K68" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi (genel misafir hattı)</t>
         </is>
       </c>
-      <c r="L68" s="12" t="inlineStr">
+      <c r="L68" s="5" t="inlineStr">
         <is>
           <t>https://gili-lankanfushi.com/contact-us/</t>
         </is>
       </c>
-      <c r="M68" s="12" t="inlineStr">
+      <c r="M68" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N68" s="12" t="n">
+      <c r="N68" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O68" s="13" t="inlineStr">
@@ -7642,75 +9060,80 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P68" s="12" t="inlineStr">
+      <c r="P68" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; GES var ama ESS yok -&gt; en uygun ESS ilavesi hedefi</t>
         </is>
       </c>
+      <c r="Q68" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="12" t="n">
+      <c r="A69" s="5" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>Grand Park Kodhipparu</t>
         </is>
       </c>
-      <c r="C69" s="12" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D69" s="12" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>Park Hotel Group</t>
         </is>
       </c>
-      <c r="E69" s="12" t="n">
+      <c r="E69" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="F69" s="12" t="inlineStr">
+      <c r="F69" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G69" s="12" t="inlineStr">
+      <c r="G69" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H69" s="12" t="inlineStr">
+      <c r="H69" s="5" t="inlineStr">
         <is>
           <t>grandparkkodhipparu.com</t>
         </is>
       </c>
-      <c r="I69" s="12" t="inlineStr">
+      <c r="I69" s="5" t="inlineStr">
         <is>
           <t>info@grandparkkodhipparu.com; rsvn.gpkd@parkhotelgroup.com</t>
         </is>
       </c>
-      <c r="J69" s="12" t="inlineStr">
+      <c r="J69" s="5" t="inlineStr">
         <is>
           <t>+960 665 1111</t>
         </is>
       </c>
-      <c r="K69" s="12" t="inlineStr">
+      <c r="K69" s="5" t="inlineStr">
         <is>
           <t>Arama sonucu</t>
         </is>
       </c>
-      <c r="L69" s="12" t="inlineStr">
+      <c r="L69" s="5" t="inlineStr">
         <is>
           <t>https://wetu.com/iBrochure/en/Information/141358/grand_park_kodhipparu/Contact</t>
         </is>
       </c>
-      <c r="M69" s="12" t="inlineStr">
+      <c r="M69" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N69" s="12" t="n">
+      <c r="N69" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O69" s="13" t="inlineStr">
@@ -7718,75 +9141,80 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P69" s="12" t="inlineStr">
+      <c r="P69" s="5" t="inlineStr">
         <is>
           <t>orta-büyük resort; bilinen GES yok -&gt; GES+ESS paketi</t>
         </is>
       </c>
+      <c r="Q69" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="12" t="n">
+      <c r="A70" s="5" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="12" t="inlineStr">
+      <c r="B70" s="5" t="inlineStr">
         <is>
           <t>InterContinental Maamunagau</t>
         </is>
       </c>
-      <c r="C70" s="12" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>Raa</t>
         </is>
       </c>
-      <c r="D70" s="12" t="inlineStr">
+      <c r="D70" s="5" t="inlineStr">
         <is>
           <t>IHG markası</t>
         </is>
       </c>
-      <c r="E70" s="12" t="n">
+      <c r="E70" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="F70" s="12" t="inlineStr">
+      <c r="F70" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G70" s="12" t="inlineStr">
+      <c r="G70" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H70" s="12" t="inlineStr">
+      <c r="H70" s="5" t="inlineStr">
         <is>
           <t>ihg.com</t>
         </is>
       </c>
-      <c r="I70" s="12" t="inlineStr">
+      <c r="I70" s="5" t="inlineStr">
         <is>
           <t>Intercontinental.Maldives@ihg.com</t>
         </is>
       </c>
-      <c r="J70" s="12" t="inlineStr">
+      <c r="J70" s="5" t="inlineStr">
         <is>
           <t>+960 658 0500</t>
         </is>
       </c>
-      <c r="K70" s="12" t="inlineStr">
+      <c r="K70" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L70" s="12" t="inlineStr">
+      <c r="L70" s="5" t="inlineStr">
         <is>
           <t>https://maldives.intercontinental.com/contact-form/</t>
         </is>
       </c>
-      <c r="M70" s="12" t="inlineStr">
+      <c r="M70" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N70" s="12" t="n">
+      <c r="N70" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O70" s="13" t="inlineStr">
@@ -7794,75 +9222,80 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P70" s="12" t="inlineStr">
+      <c r="P70" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
         </is>
       </c>
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="12" t="n">
+      <c r="A71" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="12" t="inlineStr">
+      <c r="B71" s="5" t="inlineStr">
         <is>
           <t>Kandolhu Maldives</t>
         </is>
       </c>
-      <c r="C71" s="12" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>Alif Alif (Kuzey Ari)</t>
         </is>
       </c>
-      <c r="D71" s="12" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>VERSA Hospitality</t>
         </is>
       </c>
-      <c r="E71" s="12" t="n">
+      <c r="E71" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="F71" s="12" t="inlineStr">
+      <c r="F71" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G71" s="12" t="inlineStr">
+      <c r="G71" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H71" s="12" t="inlineStr">
+      <c r="H71" s="5" t="inlineStr">
         <is>
           <t>kandolhu.com</t>
         </is>
       </c>
-      <c r="I71" s="12" t="inlineStr">
+      <c r="I71" s="5" t="inlineStr">
         <is>
           <t>info@kandolhu.com</t>
         </is>
       </c>
-      <c r="J71" s="12" t="inlineStr">
+      <c r="J71" s="5" t="inlineStr">
         <is>
           <t>+960 668 0790</t>
         </is>
       </c>
-      <c r="K71" s="12" t="inlineStr">
+      <c r="K71" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L71" s="12" t="inlineStr">
+      <c r="L71" s="5" t="inlineStr">
         <is>
           <t>https://www.kandolhu.com/contact.html</t>
         </is>
       </c>
-      <c r="M71" s="12" t="inlineStr">
+      <c r="M71" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N71" s="12" t="n">
+      <c r="N71" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O71" s="13" t="inlineStr">
@@ -7870,9 +9303,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P71" s="12" t="inlineStr">
+      <c r="P71" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q71" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -7953,68 +9391,68 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="12" t="n">
+      <c r="A73" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="B73" s="12" t="inlineStr">
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>Milaidhoo Maldives</t>
         </is>
       </c>
-      <c r="C73" s="12" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>Baa</t>
         </is>
       </c>
-      <c r="D73" s="12" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>VERSA Hospitality</t>
         </is>
       </c>
-      <c r="E73" s="12" t="n">
+      <c r="E73" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="F73" s="12" t="inlineStr">
+      <c r="F73" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G73" s="12" t="inlineStr">
+      <c r="G73" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H73" s="12" t="inlineStr">
+      <c r="H73" s="5" t="inlineStr">
         <is>
           <t>milaidhoo.com</t>
         </is>
       </c>
-      <c r="I73" s="12" t="inlineStr">
+      <c r="I73" s="5" t="inlineStr">
         <is>
           <t>welcome@milaidhoo.com</t>
         </is>
       </c>
-      <c r="J73" s="12" t="inlineStr">
+      <c r="J73" s="5" t="inlineStr">
         <is>
           <t>+960 660 7788</t>
         </is>
       </c>
-      <c r="K73" s="12" t="inlineStr">
+      <c r="K73" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi (Universal Enterprises / VERSA)</t>
         </is>
       </c>
-      <c r="L73" s="12" t="inlineStr">
+      <c r="L73" s="5" t="inlineStr">
         <is>
           <t>https://www.milaidhoo.com/contact-us.html</t>
         </is>
       </c>
-      <c r="M73" s="12" t="inlineStr">
+      <c r="M73" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N73" s="12" t="n">
+      <c r="N73" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O73" s="13" t="inlineStr">
@@ -8022,75 +9460,80 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P73" s="12" t="inlineStr">
+      <c r="P73" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
         </is>
       </c>
+      <c r="Q73" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="12" t="n">
+      <c r="A74" s="5" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="12" t="inlineStr">
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>Reethi Beach Resort</t>
         </is>
       </c>
-      <c r="C74" s="12" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>Baa</t>
         </is>
       </c>
-      <c r="D74" s="12" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>NH Collection (Minor Hotels)</t>
         </is>
       </c>
-      <c r="E74" s="12" t="n">
+      <c r="E74" s="5" t="n">
         <v>115</v>
       </c>
-      <c r="F74" s="12" t="inlineStr">
+      <c r="F74" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G74" s="12" t="inlineStr">
+      <c r="G74" s="5" t="inlineStr">
         <is>
           <t>Yeni adı NH Collection Maldives Reethi</t>
         </is>
       </c>
-      <c r="H74" s="12" t="inlineStr">
+      <c r="H74" s="5" t="inlineStr">
         <is>
           <t>nh-collection.com</t>
         </is>
       </c>
-      <c r="I74" s="12" t="inlineStr">
+      <c r="I74" s="5" t="inlineStr">
         <is>
           <t>reethi@nhcollection.com</t>
         </is>
       </c>
-      <c r="J74" s="12" t="inlineStr">
+      <c r="J74" s="5" t="inlineStr">
         <is>
           <t>+960 660 2626</t>
         </is>
       </c>
-      <c r="K74" s="12" t="inlineStr">
+      <c r="K74" s="5" t="inlineStr">
         <is>
           <t>NOT: Yeni adı 'NH Collection Maldives Reethi Resort' (Minor/NH)</t>
         </is>
       </c>
-      <c r="L74" s="12" t="inlineStr">
+      <c r="L74" s="5" t="inlineStr">
         <is>
           <t>https://www.hotelcontact.net/reethi-beach-resort-maldives-baa-en.html</t>
         </is>
       </c>
-      <c r="M74" s="12" t="inlineStr">
+      <c r="M74" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N74" s="12" t="n">
+      <c r="N74" s="5" t="n">
         <v>4</v>
       </c>
       <c r="O74" s="13" t="inlineStr">
@@ -8098,9 +9541,14 @@
           <t>B</t>
         </is>
       </c>
-      <c r="P74" s="12" t="inlineStr">
+      <c r="P74" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi; çok-resortlu grup (tek kararla birden fazla ada)</t>
+        </is>
+      </c>
+      <c r="Q74" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -8333,68 +9781,68 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="12" t="n">
+      <c r="A78" s="5" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="12" t="inlineStr">
+      <c r="B78" s="5" t="inlineStr">
         <is>
           <t>Biyadhoo Island Resort</t>
         </is>
       </c>
-      <c r="C78" s="12" t="inlineStr">
+      <c r="C78" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Güney Malé)</t>
         </is>
       </c>
-      <c r="D78" s="12" t="inlineStr">
+      <c r="D78" s="5" t="inlineStr">
         <is>
           <t>Bağımsız</t>
         </is>
       </c>
-      <c r="E78" s="12" t="n">
+      <c r="E78" s="5" t="n">
         <v>96</v>
       </c>
-      <c r="F78" s="12" t="inlineStr">
+      <c r="F78" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G78" s="12" t="inlineStr">
+      <c r="G78" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H78" s="12" t="inlineStr">
+      <c r="H78" s="5" t="inlineStr">
         <is>
           <t>biyadhoo.com</t>
         </is>
       </c>
-      <c r="I78" s="12" t="inlineStr">
+      <c r="I78" s="5" t="inlineStr">
         <is>
           <t>biyadhoo@sunland.com.mv</t>
         </is>
       </c>
-      <c r="J78" s="12" t="inlineStr">
+      <c r="J78" s="5" t="inlineStr">
         <is>
           <t>+960 664 7171</t>
         </is>
       </c>
-      <c r="K78" s="12" t="inlineStr">
+      <c r="K78" s="5" t="inlineStr">
         <is>
           <t>Arama sonucu (Sunland grubu)</t>
         </is>
       </c>
-      <c r="L78" s="12" t="inlineStr">
+      <c r="L78" s="5" t="inlineStr">
         <is>
           <t>https://www.tripadvisor.com/ShowTopic-g298335-i9918-k6983585-How_to_contact_Biyadhoo_Island_Resort_in_Maldives-South_Male_Atoll.html</t>
         </is>
       </c>
-      <c r="M78" s="12" t="inlineStr">
+      <c r="M78" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N78" s="12" t="n">
+      <c r="N78" s="5" t="n">
         <v>3</v>
       </c>
       <c r="O78" s="14" t="inlineStr">
@@ -8402,75 +9850,80 @@
           <t>C</t>
         </is>
       </c>
-      <c r="P78" s="12" t="inlineStr">
+      <c r="P78" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi</t>
         </is>
       </c>
+      <c r="Q78" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="12" t="n">
+      <c r="A79" s="5" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="12" t="inlineStr">
+      <c r="B79" s="5" t="inlineStr">
         <is>
           <t>Malahini Kuda Bandos</t>
         </is>
       </c>
-      <c r="C79" s="12" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D79" s="12" t="inlineStr">
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t>Bağımsız</t>
         </is>
       </c>
-      <c r="E79" s="12" t="n">
+      <c r="E79" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="F79" s="12" t="inlineStr">
+      <c r="F79" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G79" s="12" t="inlineStr">
+      <c r="G79" s="5" t="inlineStr">
         <is>
           <t>Akademik GES+ESS fizibilite çalışmasına konu oldu</t>
         </is>
       </c>
-      <c r="H79" s="12" t="inlineStr">
+      <c r="H79" s="5" t="inlineStr">
         <is>
           <t>malahini.com</t>
         </is>
       </c>
-      <c r="I79" s="12" t="inlineStr">
+      <c r="I79" s="5" t="inlineStr">
         <is>
           <t>reservations@malahini.mv</t>
         </is>
       </c>
-      <c r="J79" s="12" t="inlineStr">
+      <c r="J79" s="5" t="inlineStr">
         <is>
           <t>+960 664 4556</t>
         </is>
       </c>
-      <c r="K79" s="12" t="inlineStr">
+      <c r="K79" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi (malahini.mv)</t>
         </is>
       </c>
-      <c r="L79" s="12" t="inlineStr">
+      <c r="L79" s="5" t="inlineStr">
         <is>
           <t>https://malahini.mv/</t>
         </is>
       </c>
-      <c r="M79" s="12" t="inlineStr">
+      <c r="M79" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N79" s="12" t="n">
+      <c r="N79" s="5" t="n">
         <v>3</v>
       </c>
       <c r="O79" s="14" t="inlineStr">
@@ -8478,75 +9931,80 @@
           <t>C</t>
         </is>
       </c>
-      <c r="P79" s="12" t="inlineStr">
+      <c r="P79" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi</t>
         </is>
       </c>
+      <c r="Q79" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="12" t="n">
+      <c r="A80" s="5" t="n">
         <v>79</v>
       </c>
-      <c r="B80" s="12" t="inlineStr">
+      <c r="B80" s="5" t="inlineStr">
         <is>
           <t>Summer Island Maldives</t>
         </is>
       </c>
-      <c r="C80" s="12" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr">
         <is>
           <t>Kaafu (Kuzey Malé)</t>
         </is>
       </c>
-      <c r="D80" s="12" t="inlineStr">
+      <c r="D80" s="5" t="inlineStr">
         <is>
           <t>Bağımsız</t>
         </is>
       </c>
-      <c r="E80" s="12" t="n">
+      <c r="E80" s="5" t="n">
         <v>110</v>
       </c>
-      <c r="F80" s="12" t="inlineStr">
+      <c r="F80" s="5" t="inlineStr">
         <is>
           <t>Dizel ağırlıklı (kamuya açık GES bilgisi yok)</t>
         </is>
       </c>
-      <c r="G80" s="12" t="inlineStr">
+      <c r="G80" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H80" s="12" t="inlineStr">
+      <c r="H80" s="5" t="inlineStr">
         <is>
           <t>summerislandmaldives.com</t>
         </is>
       </c>
-      <c r="I80" s="12" t="inlineStr">
+      <c r="I80" s="5" t="inlineStr">
         <is>
           <t>reservations@summerislandmaldives.com</t>
         </is>
       </c>
-      <c r="J80" s="12" t="inlineStr">
+      <c r="J80" s="5" t="inlineStr">
         <is>
           <t>+960 664 1949</t>
         </is>
       </c>
-      <c r="K80" s="12" t="inlineStr">
+      <c r="K80" s="5" t="inlineStr">
         <is>
           <t>Otelin kendi sitesi</t>
         </is>
       </c>
-      <c r="L80" s="12" t="inlineStr">
+      <c r="L80" s="5" t="inlineStr">
         <is>
           <t>https://www.summerislandmaldives.com/contact-us</t>
         </is>
       </c>
-      <c r="M80" s="12" t="inlineStr">
+      <c r="M80" s="5" t="inlineStr">
         <is>
           <t>Resort: Director of Engineering / Chief Engineer, General Manager; Grup: Technical Services / Sustainability Director</t>
         </is>
       </c>
-      <c r="N80" s="12" t="n">
+      <c r="N80" s="5" t="n">
         <v>3</v>
       </c>
       <c r="O80" s="14" t="inlineStr">
@@ -8554,9 +10012,14 @@
           <t>C</t>
         </is>
       </c>
-      <c r="P80" s="12" t="inlineStr">
+      <c r="P80" s="5" t="inlineStr">
         <is>
           <t>küçük/butik resort; bilinen GES yok -&gt; GES+ESS paketi</t>
+        </is>
+      </c>
+      <c r="Q80" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -10228,32 +11691,32 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Centara Hotels &amp; Resorts</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Bangkok, Tayland</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>3+</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Machchafushi (eski Centara Grand), Ras Fushi, Mirage Lagoon</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Machchafushi'de çatı GES -&gt; ESS ilavesi</t>
         </is>
       </c>
-      <c r="F14" s="12" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>centarahotelsresorts.com</t>
         </is>
@@ -10263,24 +11726,29 @@
           <t>B</t>
         </is>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I14" s="12" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J14" s="12" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K14" s="12" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Türk sahipli yeni hedefler (Gürok/JOALI, Astaş, Maxx Royal) gruplara eklendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vs3tis47Aza7HeP1K6EeuU
</commit_message>
<xml_diff>
--- a/Maldivler_Potansiyel_Musteri_Listesi.xlsx
+++ b/Maldivler_Potansiyel_Musteri_Listesi.xlsx
@@ -252,8 +252,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Gruplar" displayName="Gruplar" ref="A1:L18" headerRowCount="1">
-  <autoFilter ref="A1:L18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Gruplar" displayName="Gruplar" ref="A1:L21" headerRowCount="1">
+  <autoFilter ref="A1:L21"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Grup"/>
     <tableColumn id="2" name="Merkez"/>
@@ -10877,7 +10877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -11381,220 +11381,205 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Aitken Spence (Adaaran / Heritance)</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Colombo, Sri Lanka</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Adaaran Hudhuranfushi, Rannalhi, Vadoo, Heritance Aarah</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Kamuya açık GES bilgisi sınırlı</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>aitkenspencehotels.com</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>inquiries.mv@adaaran.com.mv</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>+960 664 0375</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>H. Thuniya 6. kat, Boduthakurufaanu Magu, Malé 20026</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>https://www.aitkenspencehotels.com/contact-us.html</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>Mail gönderildi (2026-10-06)</t>
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Gürok Grubu (TÜRK – JOALI sahibi)</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Kütahya, Türkiye</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>JOALI Maldives, JOALI BEING (Raa Atoll)</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Ultra lüks, sürdürülebilirlik odaklı; kamuya açık GES bilgisi yok. Türk sahipli – Türkçe görüşme</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>gurok.com</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>info@gurok.com</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>+90 274 225 06 60</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>İnköy Mah. Eskişehir Karayolu Blv. No:96, Kütahya</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>https://gurok.com/iletisim</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Cinnamon Hotels (John Keells)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Colombo, Sri Lanka</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Dhonveli, Velifushi, Ellaidhoo, Hakuraa</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Kamuya açık GES bilgisi sınırlı</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>cinnamonhotels.com</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>sales.mv@cinnamonhotels.com</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>+960 333 6000</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>H. Maizan Building 2. kat, Sosun Magu, Malé 20252</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>https://www.maldivesyp.com/company/547/Cinnamon_Dhonveli_Maldives</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>Mail gönderildi (2026-10-06)</t>
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Astaş Holding (TÜRK – yeni Maldivler projesi)</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>İstanbul, Türkiye</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Proje</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>~120 villalık, 300 M$ resort projesi (Mandarin Oriental Bodrum sahibi)</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Tasarım aşamasında – enerji sistemi baştan hibrit kurgulanabilir. EN SICAK yeni proje adayı</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>astas-holding.com</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>info@astas-holding.com</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>+90 212 215 20 20</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Büyükdere Cad. No:127 Astoria Kuleleri B Blok K:25, Esentepe, İstanbul</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>https://www.astas-holding.com/tr/iletisim</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Minor Hotels (Anantara, NH Collection)</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Bangkok, Tayland</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>5+</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Anantara Dhigu/Veli/Naladhu, Kihavah, NH Reethi</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Kamuya açık GES bilgisi sınırlı. Malé adresi VERSA ile aynı – adaların sahibi VERSA olabilir (doğrulanmalı)</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>minorhotels.com</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>reservations.maldives@anantara.com</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>+960 664 4123</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>39 Orchid Magu, Malé (VERSA ile aynı adres – mülk sahipliği bağlantısı doğrulanmalı)</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>https://www.minorhotels.com/en/reservations-offices</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>Mail gönderildi (2026-10-06)</t>
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Maxx Royal Resorts (TÜRK – Maxx Royal Maldives)</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Antalya / Bodrum, Türkiye</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Proje</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Maxx Royal Maldives (5 ada, 2027 açılış hedefi)</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Yapım/tasarım aşamasında – enerji sistemi baştan hibrit kurgulanabilir</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>maxxroyal.com</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>contact@maxxroyal.com</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>+90 252 311 01 50</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Bodrum ofisi</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>https://www.maxxroyal.com/contact</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Pulse Hotels &amp; Resorts (Kandima)</t>
+          <t>Aitken Spence (Adaaran / Heritance)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Malé / Singapur</t>
+          <t>Colombo, Sri Lanka</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Kandima</t>
+          <t>Adaaran Hudhuranfushi, Rannalhi, Vadoo, Heritance Aarah</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Kamuya açık GES bilgisi yok. Mayıs 2026'da Director of Engineering ilanı açtı (yeni kişi göreve başlamış olabilir)</t>
+          <t>Kamuya açık GES bilgisi sınırlı</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>kandima.com</t>
+          <t>aitkenspencehotels.com</t>
         </is>
       </c>
       <c r="G12" s="13" t="inlineStr">
@@ -11604,22 +11589,22 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>KeepinTouch@pulseresorts.com</t>
+          <t>inquiries.mv@adaaran.com.mv</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>+65 6838 9123 (Singapur)</t>
+          <t>+960 664 0375</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Kaneeru Villa 4. kat, Orchid Magu, Malé 20212</t>
+          <t>H. Thuniya 6. kat, Boduthakurufaanu Magu, Malé 20026</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>https://kandima.com/en/explore/contact</t>
+          <t>https://www.aitkenspencehotels.com/contact-us.html</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -11631,32 +11616,32 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>CROSSROADS / Singha Estate</t>
+          <t>Cinnamon Hotels (John Keells)</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Bangkok, Tayland</t>
+          <t>Colombo, Sri Lanka</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>2 + marina</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Hard Rock, SAii Lagoon</t>
+          <t>Dhonveli, Velifushi, Ellaidhoo, Hakuraa</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Entegre ada kompleksi, tek enerji santrali</t>
+          <t>Kamuya açık GES bilgisi sınırlı</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>crossroadsmaldives.com</t>
+          <t>cinnamonhotels.com</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
@@ -11666,22 +11651,22 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>sales@crossroadsmaldives.com</t>
+          <t>sales.mv@cinnamonhotels.com</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>+960 665 1200</t>
+          <t>+960 333 6000</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>South Malé Atoll, P.O. Box 2097</t>
+          <t>H. Maizan Building 2. kat, Sosun Magu, Malé 20252</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>https://crossroadsmaldives.com/contact-us/</t>
+          <t>https://www.maldivesyp.com/company/547/Cinnamon_Dhonveli_Maldives</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
@@ -11693,7 +11678,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Centara Hotels &amp; Resorts</t>
+          <t>Minor Hotels (Anantara, NH Collection)</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -11703,22 +11688,22 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>3+</t>
+          <t>5+</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Machchafushi (eski Centara Grand), Ras Fushi, Mirage Lagoon</t>
+          <t>Anantara Dhigu/Veli/Naladhu, Kihavah, NH Reethi</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Machchafushi'de çatı GES -&gt; ESS ilavesi</t>
+          <t>Kamuya açık GES bilgisi sınırlı. Malé adresi VERSA ile aynı – adaların sahibi VERSA olabilir (doğrulanmalı)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>centarahotelsresorts.com</t>
+          <t>minorhotels.com</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
@@ -11728,22 +11713,22 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>reservations.maldives@anantara.com</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+960 664 4123</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>39 Orchid Magu, Malé (VERSA ile aynı adres – mülk sahipliği bağlantısı doğrulanmalı)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>https://www.minorhotels.com/en/reservations-offices</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
@@ -11755,231 +11740,417 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>Pulse Hotels &amp; Resorts (Kandima)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Malé / Singapur</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Kandima</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Kamuya açık GES bilgisi yok. Mayıs 2026'da Director of Engineering ilanı açtı (yeni kişi göreve başlamış olabilir)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>kandima.com</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>KeepinTouch@pulseresorts.com</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>+65 6838 9123 (Singapur)</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Kaneeru Villa 4. kat, Orchid Magu, Malé 20212</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>https://kandima.com/en/explore/contact</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CROSSROADS / Singha Estate</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Bangkok, Tayland</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>2 + marina</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Hard Rock, SAii Lagoon</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Entegre ada kompleksi, tek enerji santrali</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>crossroadsmaldives.com</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>sales@crossroadsmaldives.com</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>+960 665 1200</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>South Malé Atoll, P.O. Box 2097</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>https://crossroadsmaldives.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Centara Hotels &amp; Resorts</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Bangkok, Tayland</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>3+</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Machchafushi (eski Centara Grand), Ras Fushi, Mirage Lagoon</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Machchafushi'de çatı GES -&gt; ESS ilavesi</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>centarahotelsresorts.com</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Mail gönderildi (2026-10-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
           <t>Emerald Collection</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Doğrulanmalı</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Emerald Maldives, Emerald Faarufushi</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Kamuya açık GES bilgisi yok</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>emerald-maldives.com</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="G18" s="13" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="L18" s="5" t="inlineStr">
         <is>
           <t>Mail gönderildi (2026-10-06)</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Pontiac Land (Fari Islands)</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Singapur</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>3 (Capella 2027)</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Patina, Ritz-Carlton, Capella</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Swimsol ile büyük GES+ESS – rakip tarafından alınmış</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>fari-islands.com</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H19" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I16" s="12" t="inlineStr">
+      <c r="I19" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J16" s="12" t="inlineStr">
+      <c r="J19" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K16" s="12" t="inlineStr">
+      <c r="K19" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Soneva</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Maldivler / Dubai</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Soneva Fushi, Jani, Secret</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Canopy Power + Huawei ESS – rakip tarafından alınmış (referans vaka)</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="F20" s="12" t="inlineStr">
         <is>
           <t>soneva.com</t>
         </is>
       </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="G20" s="14" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="H20" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I17" s="12" t="inlineStr">
+      <c r="I20" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J17" s="12" t="inlineStr">
+      <c r="J20" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K17" s="12" t="inlineStr">
+      <c r="K20" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Marriott / Hilton / IHG / Four Seasons vb. küresel markalar</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Çeşitli</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Çok sayıda</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Waldorf, Conrad, Sheraton, Holiday Inn, Four Seasons</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Karar çoğunlukla mülk sahibi (owner) şirkette; marka sadece işletmeci. Owner şirket tespit edilmeli</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
+      <c r="G21" s="13" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="H18" s="12" t="inlineStr">
+      <c r="H21" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I18" s="12" t="inlineStr">
+      <c r="I21" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J18" s="12" t="inlineStr">
+      <c r="J21" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K18" s="12" t="inlineStr">
+      <c r="K21" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>